<commit_message>
Only prevention changes SAM treatment needs
</commit_message>
<xml_diff>
--- a/tests/scen_results_AGO2.xlsx
+++ b/tests/scen_results_AGO2.xlsx
@@ -27,7 +27,7 @@
     <t>2.0.11</t>
   </si>
   <si>
-    <t>2025-04-24</t>
+    <t>2025-04-28</t>
   </si>
   <si>
     <t>Scenario</t>
@@ -23818,34 +23818,34 @@
         <v>4212219.410027994</v>
       </c>
       <c r="G82" s="3">
-        <v>4262144.492062939</v>
+        <v>4238208.375984523</v>
       </c>
       <c r="H82" s="3">
-        <v>4317444.501416235</v>
+        <v>4268730.9962528</v>
       </c>
       <c r="I82" s="3">
-        <v>4375317.305816489</v>
+        <v>4300864.898670025</v>
       </c>
       <c r="J82" s="3">
-        <v>4437294.279713682</v>
+        <v>4335994.840180334</v>
       </c>
       <c r="K82" s="3">
-        <v>4501694.940340191</v>
+        <v>4372381.349151926</v>
       </c>
       <c r="L82" s="3">
-        <v>4569437.695280578</v>
+        <v>4411376.721499375</v>
       </c>
       <c r="M82" s="3">
-        <v>4639645.162146033</v>
+        <v>4452086.777320319</v>
       </c>
       <c r="N82" s="3">
-        <v>4708793.900967901</v>
+        <v>4491131.712348624</v>
       </c>
       <c r="O82" s="3">
-        <v>4778069.337999758</v>
+        <v>4529676.327589785</v>
       </c>
       <c r="P82" s="3">
-        <v>4846841.643099741</v>
+        <v>4567130.112100023</v>
       </c>
     </row>
     <row r="83" spans="1:16">
@@ -24026,34 +24026,34 @@
         <v>5884718.293421461</v>
       </c>
       <c r="G87" s="3">
-        <v>11595599.47454362</v>
+        <v>11530478.53190138</v>
       </c>
       <c r="H87" s="3">
-        <v>17460704.7446452</v>
+        <v>17263694.1381687</v>
       </c>
       <c r="I87" s="3">
-        <v>23164806.95665973</v>
+        <v>22770616.32214574</v>
       </c>
       <c r="J87" s="3">
-        <v>29367375.01863801</v>
+        <v>28696927.35384338</v>
       </c>
       <c r="K87" s="3">
-        <v>29794997.06917733</v>
+        <v>28939094.78278884</v>
       </c>
       <c r="L87" s="3">
-        <v>30244449.92030663</v>
+        <v>29198235.93966736</v>
       </c>
       <c r="M87" s="3">
-        <v>30709955.55400643</v>
+        <v>29468466.5486116</v>
       </c>
       <c r="N87" s="3">
-        <v>31168246.54063012</v>
+        <v>29727471.80631435</v>
       </c>
       <c r="O87" s="3">
-        <v>31627217.21562619</v>
+        <v>29983010.13487854</v>
       </c>
       <c r="P87" s="3">
-        <v>32082742.53366321</v>
+        <v>30231216.48272794</v>
       </c>
     </row>
     <row r="88" spans="1:16">

</xml_diff>